<commit_message>
Update - Final version
</commit_message>
<xml_diff>
--- a/output/step4_exposure_instability_matrix.xlsx
+++ b/output/step4_exposure_instability_matrix.xlsx
@@ -28,7 +28,7 @@
     <t>Pct_anomalous_months</t>
   </si>
   <si>
-    <t>Average_intensity_recency_weighted</t>
+    <t>Average_intensity_recency_severity_weighted</t>
   </si>
   <si>
     <t>KPI_level</t>
@@ -526,7 +526,7 @@
         <v>16.76</v>
       </c>
       <c r="E2">
-        <v>5.05</v>
+        <v>6.17</v>
       </c>
       <c r="F2">
         <v>2</v>
@@ -538,7 +538,7 @@
         <v>2.56</v>
       </c>
       <c r="I2">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J2" t="s">
         <v>40</v>
@@ -558,7 +558,7 @@
         <v>14.05</v>
       </c>
       <c r="E3">
-        <v>5.63</v>
+        <v>6.91</v>
       </c>
       <c r="F3">
         <v>2</v>
@@ -570,7 +570,7 @@
         <v>2.56</v>
       </c>
       <c r="I3">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J3" t="s">
         <v>41</v>
@@ -590,7 +590,7 @@
         <v>13.51</v>
       </c>
       <c r="E4">
-        <v>5.95</v>
+        <v>7.47</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -602,7 +602,7 @@
         <v>2.56</v>
       </c>
       <c r="I4">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J4" t="s">
         <v>41</v>
@@ -622,7 +622,7 @@
         <v>16.76</v>
       </c>
       <c r="E5">
-        <v>6.83</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -634,7 +634,7 @@
         <v>2.56</v>
       </c>
       <c r="I5">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J5" t="s">
         <v>41</v>
@@ -654,7 +654,7 @@
         <v>16.76</v>
       </c>
       <c r="E6">
-        <v>4.1</v>
+        <v>4.68</v>
       </c>
       <c r="F6">
         <v>3</v>
@@ -666,7 +666,7 @@
         <v>2.56</v>
       </c>
       <c r="I6">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J6" t="s">
         <v>40</v>
@@ -686,7 +686,7 @@
         <v>11.35</v>
       </c>
       <c r="E7">
-        <v>5.22</v>
+        <v>6.55</v>
       </c>
       <c r="F7">
         <v>3</v>
@@ -698,7 +698,7 @@
         <v>2.56</v>
       </c>
       <c r="I7">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J7" t="s">
         <v>40</v>
@@ -718,7 +718,7 @@
         <v>18.92</v>
       </c>
       <c r="E8">
-        <v>6.09</v>
+        <v>7.54</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -730,7 +730,7 @@
         <v>2.56</v>
       </c>
       <c r="I8">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J8" t="s">
         <v>42</v>
@@ -750,7 +750,7 @@
         <v>12.97</v>
       </c>
       <c r="E9">
-        <v>5.88</v>
+        <v>6.66</v>
       </c>
       <c r="F9">
         <v>1</v>
@@ -762,7 +762,7 @@
         <v>2.56</v>
       </c>
       <c r="I9">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J9" t="s">
         <v>42</v>
@@ -782,7 +782,7 @@
         <v>17.3</v>
       </c>
       <c r="E10">
-        <v>7.05</v>
+        <v>8.58</v>
       </c>
       <c r="F10">
         <v>1</v>
@@ -794,7 +794,7 @@
         <v>2.56</v>
       </c>
       <c r="I10">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J10" t="s">
         <v>42</v>
@@ -814,7 +814,7 @@
         <v>12.97</v>
       </c>
       <c r="E11">
-        <v>7.72</v>
+        <v>8.59</v>
       </c>
       <c r="F11">
         <v>1</v>
@@ -826,7 +826,7 @@
         <v>2.56</v>
       </c>
       <c r="I11">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J11" t="s">
         <v>42</v>
@@ -846,7 +846,7 @@
         <v>14.59</v>
       </c>
       <c r="E12">
-        <v>4.5</v>
+        <v>5.64</v>
       </c>
       <c r="F12">
         <v>1</v>
@@ -858,7 +858,7 @@
         <v>2.56</v>
       </c>
       <c r="I12">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J12" t="s">
         <v>43</v>
@@ -878,7 +878,7 @@
         <v>14.05</v>
       </c>
       <c r="E13">
-        <v>8.77</v>
+        <v>10.45</v>
       </c>
       <c r="F13">
         <v>1</v>
@@ -890,7 +890,7 @@
         <v>2.56</v>
       </c>
       <c r="I13">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J13" t="s">
         <v>42</v>
@@ -910,7 +910,7 @@
         <v>17.84</v>
       </c>
       <c r="E14">
-        <v>3.32</v>
+        <v>4.05</v>
       </c>
       <c r="F14">
         <v>3</v>
@@ -922,7 +922,7 @@
         <v>2.56</v>
       </c>
       <c r="I14">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J14" t="s">
         <v>43</v>
@@ -942,7 +942,7 @@
         <v>16.22</v>
       </c>
       <c r="E15">
-        <v>4.77</v>
+        <v>5.66</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -954,7 +954,7 @@
         <v>2.56</v>
       </c>
       <c r="I15">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J15" t="s">
         <v>43</v>
@@ -974,7 +974,7 @@
         <v>12.43</v>
       </c>
       <c r="E16">
-        <v>4.08</v>
+        <v>4.6</v>
       </c>
       <c r="F16">
         <v>2</v>
@@ -986,7 +986,7 @@
         <v>2.56</v>
       </c>
       <c r="I16">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J16" t="s">
         <v>43</v>
@@ -1006,13 +1006,13 @@
         <v>10.81</v>
       </c>
       <c r="E17">
-        <v>4.76</v>
+        <v>5.53</v>
       </c>
       <c r="H17">
         <v>2.56</v>
       </c>
       <c r="I17">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J17" t="s">
         <v>43</v>
@@ -1032,7 +1032,7 @@
         <v>14.05</v>
       </c>
       <c r="E18">
-        <v>4.24</v>
+        <v>5.12</v>
       </c>
       <c r="F18">
         <v>3</v>
@@ -1044,7 +1044,7 @@
         <v>2.56</v>
       </c>
       <c r="I18">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J18" t="s">
         <v>43</v>
@@ -1064,7 +1064,7 @@
         <v>12</v>
       </c>
       <c r="E19">
-        <v>9.390000000000001</v>
+        <v>11.78</v>
       </c>
       <c r="F19">
         <v>2</v>
@@ -1076,7 +1076,7 @@
         <v>2.56</v>
       </c>
       <c r="I19">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J19" t="s">
         <v>42</v>
@@ -1096,7 +1096,7 @@
         <v>18.92</v>
       </c>
       <c r="E20">
-        <v>9.24</v>
+        <v>10.52</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -1108,7 +1108,7 @@
         <v>2.56</v>
       </c>
       <c r="I20">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J20" t="s">
         <v>42</v>
@@ -1128,7 +1128,7 @@
         <v>20.8</v>
       </c>
       <c r="E21">
-        <v>6.23</v>
+        <v>7.61</v>
       </c>
       <c r="G21" t="s">
         <v>39</v>
@@ -1137,7 +1137,7 @@
         <v>2.56</v>
       </c>
       <c r="I21">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J21" t="s">
         <v>42</v>
@@ -1157,7 +1157,7 @@
         <v>12.97</v>
       </c>
       <c r="E22">
-        <v>13.44</v>
+        <v>16.13</v>
       </c>
       <c r="F22">
         <v>2</v>
@@ -1169,7 +1169,7 @@
         <v>2.56</v>
       </c>
       <c r="I22">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J22" t="s">
         <v>42</v>
@@ -1189,7 +1189,7 @@
         <v>15.2</v>
       </c>
       <c r="E23">
-        <v>6.24</v>
+        <v>7.78</v>
       </c>
       <c r="F23">
         <v>1</v>
@@ -1201,7 +1201,7 @@
         <v>2.56</v>
       </c>
       <c r="I23">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J23" t="s">
         <v>42</v>
@@ -1221,7 +1221,7 @@
         <v>21.62</v>
       </c>
       <c r="E24">
-        <v>4.74</v>
+        <v>5.36</v>
       </c>
       <c r="F24">
         <v>1</v>
@@ -1233,7 +1233,7 @@
         <v>2.56</v>
       </c>
       <c r="I24">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J24" t="s">
         <v>43</v>
@@ -1253,7 +1253,7 @@
         <v>14.59</v>
       </c>
       <c r="E25">
-        <v>5.01</v>
+        <v>6.31</v>
       </c>
       <c r="F25">
         <v>1</v>
@@ -1265,7 +1265,7 @@
         <v>2.56</v>
       </c>
       <c r="I25">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J25" t="s">
         <v>43</v>
@@ -1285,7 +1285,7 @@
         <v>15.14</v>
       </c>
       <c r="E26">
-        <v>3.71</v>
+        <v>4.42</v>
       </c>
       <c r="F26">
         <v>2</v>
@@ -1297,7 +1297,7 @@
         <v>2.56</v>
       </c>
       <c r="I26">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J26" t="s">
         <v>43</v>
@@ -1317,7 +1317,7 @@
         <v>16.76</v>
       </c>
       <c r="E27">
-        <v>5.05</v>
+        <v>6.17</v>
       </c>
       <c r="F27">
         <v>2</v>
@@ -1329,7 +1329,7 @@
         <v>3.36</v>
       </c>
       <c r="I27">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J27" t="s">
         <v>40</v>
@@ -1349,7 +1349,7 @@
         <v>16.76</v>
       </c>
       <c r="E28">
-        <v>6.83</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F28">
         <v>1</v>
@@ -1361,7 +1361,7 @@
         <v>3.36</v>
       </c>
       <c r="I28">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J28" t="s">
         <v>41</v>
@@ -1381,7 +1381,7 @@
         <v>13.51</v>
       </c>
       <c r="E29">
-        <v>5.95</v>
+        <v>7.47</v>
       </c>
       <c r="F29">
         <v>1</v>
@@ -1393,7 +1393,7 @@
         <v>3.36</v>
       </c>
       <c r="I29">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J29" t="s">
         <v>41</v>
@@ -1413,7 +1413,7 @@
         <v>14.05</v>
       </c>
       <c r="E30">
-        <v>5.63</v>
+        <v>6.91</v>
       </c>
       <c r="F30">
         <v>2</v>
@@ -1425,7 +1425,7 @@
         <v>3.36</v>
       </c>
       <c r="I30">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J30" t="s">
         <v>41</v>
@@ -1445,7 +1445,7 @@
         <v>16.76</v>
       </c>
       <c r="E31">
-        <v>4.1</v>
+        <v>4.68</v>
       </c>
       <c r="F31">
         <v>3</v>
@@ -1457,7 +1457,7 @@
         <v>3.36</v>
       </c>
       <c r="I31">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J31" t="s">
         <v>40</v>
@@ -1477,7 +1477,7 @@
         <v>12.97</v>
       </c>
       <c r="E32">
-        <v>5.88</v>
+        <v>6.66</v>
       </c>
       <c r="F32">
         <v>1</v>
@@ -1489,7 +1489,7 @@
         <v>3.36</v>
       </c>
       <c r="I32">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J32" t="s">
         <v>41</v>
@@ -1509,7 +1509,7 @@
         <v>11.35</v>
       </c>
       <c r="E33">
-        <v>5.22</v>
+        <v>6.55</v>
       </c>
       <c r="F33">
         <v>3</v>
@@ -1521,7 +1521,7 @@
         <v>3.36</v>
       </c>
       <c r="I33">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J33" t="s">
         <v>40</v>
@@ -1541,7 +1541,7 @@
         <v>18.92</v>
       </c>
       <c r="E34">
-        <v>6.09</v>
+        <v>7.54</v>
       </c>
       <c r="F34">
         <v>1</v>
@@ -1553,7 +1553,7 @@
         <v>3.36</v>
       </c>
       <c r="I34">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J34" t="s">
         <v>41</v>
@@ -1573,7 +1573,7 @@
         <v>14.59</v>
       </c>
       <c r="E35">
-        <v>4.5</v>
+        <v>5.64</v>
       </c>
       <c r="F35">
         <v>1</v>
@@ -1585,7 +1585,7 @@
         <v>3.36</v>
       </c>
       <c r="I35">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J35" t="s">
         <v>43</v>
@@ -1605,7 +1605,7 @@
         <v>14.05</v>
       </c>
       <c r="E36">
-        <v>8.77</v>
+        <v>10.45</v>
       </c>
       <c r="F36">
         <v>1</v>
@@ -1617,7 +1617,7 @@
         <v>3.36</v>
       </c>
       <c r="I36">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J36" t="s">
         <v>42</v>
@@ -1637,7 +1637,7 @@
         <v>16.22</v>
       </c>
       <c r="E37">
-        <v>4.77</v>
+        <v>5.66</v>
       </c>
       <c r="F37">
         <v>1</v>
@@ -1649,7 +1649,7 @@
         <v>3.36</v>
       </c>
       <c r="I37">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J37" t="s">
         <v>43</v>
@@ -1669,7 +1669,7 @@
         <v>12</v>
       </c>
       <c r="E38">
-        <v>9.390000000000001</v>
+        <v>11.78</v>
       </c>
       <c r="F38">
         <v>2</v>
@@ -1681,7 +1681,7 @@
         <v>3.36</v>
       </c>
       <c r="I38">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J38" t="s">
         <v>42</v>
@@ -1701,7 +1701,7 @@
         <v>12.97</v>
       </c>
       <c r="E39">
-        <v>7.72</v>
+        <v>8.59</v>
       </c>
       <c r="F39">
         <v>1</v>
@@ -1713,7 +1713,7 @@
         <v>3.36</v>
       </c>
       <c r="I39">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J39" t="s">
         <v>42</v>
@@ -1733,7 +1733,7 @@
         <v>17.84</v>
       </c>
       <c r="E40">
-        <v>3.32</v>
+        <v>4.05</v>
       </c>
       <c r="F40">
         <v>3</v>
@@ -1745,7 +1745,7 @@
         <v>3.36</v>
       </c>
       <c r="I40">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J40" t="s">
         <v>43</v>
@@ -1765,7 +1765,7 @@
         <v>17.3</v>
       </c>
       <c r="E41">
-        <v>7.05</v>
+        <v>8.58</v>
       </c>
       <c r="F41">
         <v>1</v>
@@ -1777,7 +1777,7 @@
         <v>3.36</v>
       </c>
       <c r="I41">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J41" t="s">
         <v>42</v>
@@ -1797,7 +1797,7 @@
         <v>12.43</v>
       </c>
       <c r="E42">
-        <v>4.08</v>
+        <v>4.6</v>
       </c>
       <c r="F42">
         <v>2</v>
@@ -1809,7 +1809,7 @@
         <v>3.36</v>
       </c>
       <c r="I42">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J42" t="s">
         <v>43</v>
@@ -1829,7 +1829,7 @@
         <v>18.92</v>
       </c>
       <c r="E43">
-        <v>9.24</v>
+        <v>10.52</v>
       </c>
       <c r="F43">
         <v>1</v>
@@ -1841,7 +1841,7 @@
         <v>3.36</v>
       </c>
       <c r="I43">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J43" t="s">
         <v>42</v>
@@ -1861,7 +1861,7 @@
         <v>14.05</v>
       </c>
       <c r="E44">
-        <v>4.24</v>
+        <v>5.12</v>
       </c>
       <c r="F44">
         <v>3</v>
@@ -1873,7 +1873,7 @@
         <v>3.36</v>
       </c>
       <c r="I44">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J44" t="s">
         <v>43</v>
@@ -1893,13 +1893,13 @@
         <v>10.81</v>
       </c>
       <c r="E45">
-        <v>4.76</v>
+        <v>5.53</v>
       </c>
       <c r="H45">
         <v>3.36</v>
       </c>
       <c r="I45">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J45" t="s">
         <v>43</v>
@@ -1919,7 +1919,7 @@
         <v>20.8</v>
       </c>
       <c r="E46">
-        <v>6.23</v>
+        <v>7.61</v>
       </c>
       <c r="G46" t="s">
         <v>39</v>
@@ -1928,7 +1928,7 @@
         <v>3.36</v>
       </c>
       <c r="I46">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J46" t="s">
         <v>42</v>
@@ -1948,7 +1948,7 @@
         <v>15.2</v>
       </c>
       <c r="E47">
-        <v>6.24</v>
+        <v>7.78</v>
       </c>
       <c r="F47">
         <v>1</v>
@@ -1960,7 +1960,7 @@
         <v>3.36</v>
       </c>
       <c r="I47">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J47" t="s">
         <v>42</v>
@@ -1980,7 +1980,7 @@
         <v>12.97</v>
       </c>
       <c r="E48">
-        <v>13.44</v>
+        <v>16.13</v>
       </c>
       <c r="F48">
         <v>2</v>
@@ -1992,7 +1992,7 @@
         <v>3.36</v>
       </c>
       <c r="I48">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J48" t="s">
         <v>42</v>
@@ -2012,7 +2012,7 @@
         <v>14.59</v>
       </c>
       <c r="E49">
-        <v>5.01</v>
+        <v>6.31</v>
       </c>
       <c r="F49">
         <v>1</v>
@@ -2024,7 +2024,7 @@
         <v>3.36</v>
       </c>
       <c r="I49">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J49" t="s">
         <v>43</v>
@@ -2044,7 +2044,7 @@
         <v>21.62</v>
       </c>
       <c r="E50">
-        <v>4.74</v>
+        <v>5.36</v>
       </c>
       <c r="F50">
         <v>1</v>
@@ -2056,7 +2056,7 @@
         <v>3.36</v>
       </c>
       <c r="I50">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J50" t="s">
         <v>43</v>
@@ -2076,7 +2076,7 @@
         <v>15.14</v>
       </c>
       <c r="E51">
-        <v>3.71</v>
+        <v>4.42</v>
       </c>
       <c r="F51">
         <v>2</v>
@@ -2088,7 +2088,7 @@
         <v>3.36</v>
       </c>
       <c r="I51">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J51" t="s">
         <v>43</v>
@@ -2108,7 +2108,7 @@
         <v>16.76</v>
       </c>
       <c r="E52">
-        <v>5.05</v>
+        <v>6.17</v>
       </c>
       <c r="F52">
         <v>2</v>
@@ -2120,7 +2120,7 @@
         <v>4.4</v>
       </c>
       <c r="I52">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J52" t="s">
         <v>40</v>
@@ -2140,7 +2140,7 @@
         <v>16.76</v>
       </c>
       <c r="E53">
-        <v>6.83</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F53">
         <v>1</v>
@@ -2152,7 +2152,7 @@
         <v>4.4</v>
       </c>
       <c r="I53">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J53" t="s">
         <v>41</v>
@@ -2172,7 +2172,7 @@
         <v>13.51</v>
       </c>
       <c r="E54">
-        <v>5.95</v>
+        <v>7.47</v>
       </c>
       <c r="F54">
         <v>1</v>
@@ -2184,7 +2184,7 @@
         <v>4.4</v>
       </c>
       <c r="I54">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J54" t="s">
         <v>41</v>
@@ -2204,7 +2204,7 @@
         <v>14.05</v>
       </c>
       <c r="E55">
-        <v>5.63</v>
+        <v>6.91</v>
       </c>
       <c r="F55">
         <v>2</v>
@@ -2216,7 +2216,7 @@
         <v>4.4</v>
       </c>
       <c r="I55">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J55" t="s">
         <v>41</v>
@@ -2236,7 +2236,7 @@
         <v>16.76</v>
       </c>
       <c r="E56">
-        <v>4.1</v>
+        <v>4.68</v>
       </c>
       <c r="F56">
         <v>3</v>
@@ -2248,7 +2248,7 @@
         <v>4.4</v>
       </c>
       <c r="I56">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J56" t="s">
         <v>40</v>
@@ -2268,7 +2268,7 @@
         <v>12.97</v>
       </c>
       <c r="E57">
-        <v>5.88</v>
+        <v>6.66</v>
       </c>
       <c r="F57">
         <v>1</v>
@@ -2280,7 +2280,7 @@
         <v>4.4</v>
       </c>
       <c r="I57">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J57" t="s">
         <v>41</v>
@@ -2300,7 +2300,7 @@
         <v>18.92</v>
       </c>
       <c r="E58">
-        <v>6.09</v>
+        <v>7.54</v>
       </c>
       <c r="F58">
         <v>1</v>
@@ -2312,7 +2312,7 @@
         <v>4.4</v>
       </c>
       <c r="I58">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J58" t="s">
         <v>41</v>
@@ -2332,7 +2332,7 @@
         <v>16.22</v>
       </c>
       <c r="E59">
-        <v>4.77</v>
+        <v>5.66</v>
       </c>
       <c r="F59">
         <v>1</v>
@@ -2344,7 +2344,7 @@
         <v>4.4</v>
       </c>
       <c r="I59">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J59" t="s">
         <v>40</v>
@@ -2364,7 +2364,7 @@
         <v>14.05</v>
       </c>
       <c r="E60">
-        <v>8.77</v>
+        <v>10.45</v>
       </c>
       <c r="F60">
         <v>1</v>
@@ -2376,7 +2376,7 @@
         <v>4.4</v>
       </c>
       <c r="I60">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J60" t="s">
         <v>42</v>
@@ -2396,7 +2396,7 @@
         <v>12</v>
       </c>
       <c r="E61">
-        <v>9.390000000000001</v>
+        <v>11.78</v>
       </c>
       <c r="F61">
         <v>2</v>
@@ -2408,7 +2408,7 @@
         <v>4.4</v>
       </c>
       <c r="I61">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J61" t="s">
         <v>42</v>
@@ -2428,7 +2428,7 @@
         <v>14.59</v>
       </c>
       <c r="E62">
-        <v>4.5</v>
+        <v>5.64</v>
       </c>
       <c r="F62">
         <v>1</v>
@@ -2440,7 +2440,7 @@
         <v>4.4</v>
       </c>
       <c r="I62">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J62" t="s">
         <v>43</v>
@@ -2460,7 +2460,7 @@
         <v>11.35</v>
       </c>
       <c r="E63">
-        <v>5.22</v>
+        <v>6.55</v>
       </c>
       <c r="F63">
         <v>3</v>
@@ -2472,7 +2472,7 @@
         <v>4.4</v>
       </c>
       <c r="I63">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J63" t="s">
         <v>43</v>
@@ -2492,7 +2492,7 @@
         <v>18.92</v>
       </c>
       <c r="E64">
-        <v>9.24</v>
+        <v>10.52</v>
       </c>
       <c r="F64">
         <v>1</v>
@@ -2504,7 +2504,7 @@
         <v>4.4</v>
       </c>
       <c r="I64">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J64" t="s">
         <v>42</v>
@@ -2524,7 +2524,7 @@
         <v>12.43</v>
       </c>
       <c r="E65">
-        <v>4.08</v>
+        <v>4.6</v>
       </c>
       <c r="F65">
         <v>2</v>
@@ -2536,7 +2536,7 @@
         <v>4.4</v>
       </c>
       <c r="I65">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J65" t="s">
         <v>43</v>
@@ -2556,7 +2556,7 @@
         <v>17.84</v>
       </c>
       <c r="E66">
-        <v>3.32</v>
+        <v>4.05</v>
       </c>
       <c r="F66">
         <v>3</v>
@@ -2568,7 +2568,7 @@
         <v>4.4</v>
       </c>
       <c r="I66">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J66" t="s">
         <v>43</v>
@@ -2588,7 +2588,7 @@
         <v>12.97</v>
       </c>
       <c r="E67">
-        <v>7.72</v>
+        <v>8.59</v>
       </c>
       <c r="F67">
         <v>1</v>
@@ -2600,7 +2600,7 @@
         <v>4.4</v>
       </c>
       <c r="I67">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J67" t="s">
         <v>42</v>
@@ -2620,7 +2620,7 @@
         <v>17.3</v>
       </c>
       <c r="E68">
-        <v>7.05</v>
+        <v>8.58</v>
       </c>
       <c r="F68">
         <v>1</v>
@@ -2632,7 +2632,7 @@
         <v>4.4</v>
       </c>
       <c r="I68">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J68" t="s">
         <v>42</v>
@@ -2652,7 +2652,7 @@
         <v>14.05</v>
       </c>
       <c r="E69">
-        <v>4.24</v>
+        <v>5.12</v>
       </c>
       <c r="F69">
         <v>3</v>
@@ -2664,7 +2664,7 @@
         <v>4.4</v>
       </c>
       <c r="I69">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J69" t="s">
         <v>43</v>
@@ -2684,13 +2684,13 @@
         <v>10.81</v>
       </c>
       <c r="E70">
-        <v>4.76</v>
+        <v>5.53</v>
       </c>
       <c r="H70">
         <v>4.4</v>
       </c>
       <c r="I70">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J70" t="s">
         <v>43</v>
@@ -2710,7 +2710,7 @@
         <v>20.8</v>
       </c>
       <c r="E71">
-        <v>6.23</v>
+        <v>7.61</v>
       </c>
       <c r="G71" t="s">
         <v>39</v>
@@ -2719,7 +2719,7 @@
         <v>4.4</v>
       </c>
       <c r="I71">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J71" t="s">
         <v>42</v>
@@ -2739,7 +2739,7 @@
         <v>15.2</v>
       </c>
       <c r="E72">
-        <v>6.24</v>
+        <v>7.78</v>
       </c>
       <c r="F72">
         <v>1</v>
@@ -2751,7 +2751,7 @@
         <v>4.4</v>
       </c>
       <c r="I72">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J72" t="s">
         <v>42</v>
@@ -2771,7 +2771,7 @@
         <v>12.97</v>
       </c>
       <c r="E73">
-        <v>13.44</v>
+        <v>16.13</v>
       </c>
       <c r="F73">
         <v>2</v>
@@ -2783,7 +2783,7 @@
         <v>4.4</v>
       </c>
       <c r="I73">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J73" t="s">
         <v>42</v>
@@ -2803,7 +2803,7 @@
         <v>14.59</v>
       </c>
       <c r="E74">
-        <v>5.01</v>
+        <v>6.31</v>
       </c>
       <c r="F74">
         <v>1</v>
@@ -2815,7 +2815,7 @@
         <v>4.4</v>
       </c>
       <c r="I74">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J74" t="s">
         <v>43</v>
@@ -2835,7 +2835,7 @@
         <v>21.62</v>
       </c>
       <c r="E75">
-        <v>4.74</v>
+        <v>5.36</v>
       </c>
       <c r="F75">
         <v>1</v>
@@ -2847,7 +2847,7 @@
         <v>4.4</v>
       </c>
       <c r="I75">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J75" t="s">
         <v>43</v>
@@ -2867,7 +2867,7 @@
         <v>15.14</v>
       </c>
       <c r="E76">
-        <v>3.71</v>
+        <v>4.42</v>
       </c>
       <c r="F76">
         <v>2</v>
@@ -2879,7 +2879,7 @@
         <v>4.4</v>
       </c>
       <c r="I76">
-        <v>5.63</v>
+        <v>6.66</v>
       </c>
       <c r="J76" t="s">
         <v>43</v>

</xml_diff>